<commit_message>
Alle Song-Tabellen auf Effekt / Änderungswunsch umgestellt
- songgen.py --tabelle ohne Song füllt die Spalte "Effekt (füllt KI)" in allen
  Tabellen, ohne Code zu erzeugen (table_texts, frozen_texts): Show + Code = die
  Gestaltung der Show, Show ohne Code mit Vermerk, eingefrorener Code über die
  Zeit zugeordnet, sonst der alte Code aus "bisher (alter Code)".
- Die 23 übrigen struktur.xlsx umgestellt: bisherige Texte aus "Effektidee"
  stehen in "Änderungswunsch", Spalte C ist gefüllt.
- Skill new-song und FX-Pipeline-Plan nachgezogen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/Apt_v1/quelle/struktur.xlsx
+++ b/songs/Apt_v1/quelle/struktur.xlsx
@@ -436,15 +436,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,6 +469,7 @@
       <c r="C2" s="2" t="n">
         <v>17</v>
       </c>
+      <c r="D2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
@@ -478,6 +480,7 @@
       <c r="C3" s="2" t="n">
         <v>149</v>
       </c>
+      <c r="D3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
@@ -488,6 +491,7 @@
       <c r="C4" s="2" t="n">
         <v>0.375</v>
       </c>
+      <c r="D4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -502,20 +506,25 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Effektidee</t>
+          <t>Effekt (füllt KI)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
+          <t>Änderungswunsch</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
           <t>Energie 0-5</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>BPM pro Part</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>bisher (alter Code)</t>
         </is>
@@ -530,13 +539,19 @@
           <t>pause</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progBlack(5840, 5)</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>progBlack(5840, 5)</t>
         </is>
@@ -551,13 +566,19 @@
           <t>bassdrum intro</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progRandomLines(12885, 10, 800, true)</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>progRandomLines(12885, 10, 800, true)</t>
         </is>
@@ -572,13 +593,19 @@
           <t>verse 1</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progFullColors(12885, 15, 805)</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>progFullColors(12885, 15, 805)</t>
         </is>
@@ -593,13 +620,19 @@
           <t>chorus 1</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progSternNeu(11275, 805, 20, 5, 26, 5, true, 3)</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>progSternNeu(11275, 805, 20, 5, 26, 5, true, 3)</t>
         </is>
@@ -614,13 +647,19 @@
           <t>STOP</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progBlack(1610, 25)</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>progBlack(1610, 25)</t>
         </is>
@@ -635,13 +674,19 @@
           <t>apt apt apt</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progMatrixScanner(12890, 28, 25)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>progMatrixScanner(12890, 28, 25)</t>
         </is>
@@ -656,13 +701,19 @@
           <t>ist whatever</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progStrobo(3220, 30, 200, 255, 255, 255)</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>progStrobo(3220, 30, 200, 255, 255, 255)</t>
         </is>
@@ -677,13 +728,19 @@
           <t>verse 2</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progPalette(9665, 3, 35)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>progPalette(9665, 3, 35)</t>
         </is>
@@ -698,13 +755,19 @@
           <t>chorus 2</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progSternNeu(11275, 805, 40, 5, 26, 5, false, 4)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>progSternNeu(11275, 805, 40, 5, 26, 5, false, 4)</t>
         </is>
@@ -719,13 +782,19 @@
           <t>STOP</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progStrobo(1610, 45, 100, 255, 255, 255)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>progStrobo(1610, 45, 100, 255, 255, 255)</t>
         </is>
@@ -740,13 +809,19 @@
           <t>apt apt apt</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progStrobo(12885, 50, 400, getRandomCRGB())</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>progStrobo(12885, 50, 400, getRandomCRGB())</t>
         </is>
@@ -761,13 +836,19 @@
           <t>hey ….</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progPalette(5640, 9, 55)   (Matrix: progOutline(5640, 55, 50))</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>progPalette(5640, 9, 55)   (Matrix: progOutline(5640, 55, 50))</t>
         </is>
@@ -782,13 +863,19 @@
           <t>get ya get ya</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progStrobo(805, 60, 50, 255, 255, 255)</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>progStrobo(805, 60, 50, 255, 255, 255)</t>
         </is>
@@ -803,13 +890,19 @@
           <t>hold on</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progFastBlingBling(25770, 4, 65, 1, 15, 2500)</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>progFastBlingBling(25770, 4, 65, 1, 15, 2500)</t>
         </is>
@@ -824,13 +917,19 @@
           <t>nur vocals</t>
         </is>
       </c>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progBlack(4830, 70)</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>progBlack(4830, 70)</t>
         </is>
@@ -845,13 +944,19 @@
           <t>strobo</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progStrobo(1610, 75, 50, 255, 255, 255)</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>progStrobo(1610, 75, 50, 255, 255, 255)</t>
         </is>
@@ -866,13 +971,19 @@
           <t>chorus 5</t>
         </is>
       </c>
-      <c r="C22" s="6" t="n"/>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progSternNeu(6445, 805, 80, 5, 26, 5, true, 3)</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>progSternNeu(6445, 805, 80, 5, 26, 5, true, 3)</t>
         </is>
@@ -887,13 +998,19 @@
           <t>apt apt apt</t>
         </is>
       </c>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5">
-        <f>$C$3</f>
-        <v/>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>alter Code (handgeschrieben, läuft so in der Firmware):
+progFastBlingBling(25775, 4, 85, 1, 15, 2500)</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5">
+        <f>$C$3</f>
+        <v/>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>progFastBlingBling(25775, 4, 85, 1, 15, 2500)</t>
         </is>
@@ -913,10 +1030,10 @@
           <t>10 sek. BLACK</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="E24" t="n">
         <v>0</v>
       </c>
-      <c r="E24">
+      <c r="F24">
         <f>$C$3</f>
         <v/>
       </c>

</xml_diff>